<commit_message>
change issueDate to inspectionDate
</commit_message>
<xml_diff>
--- a/src/main/resources/assets/template/ImportBinEntryTemplate.xlsx
+++ b/src/main/resources/assets/template/ImportBinEntryTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Backend\kvc-wh-be\src\main\resources\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E0FA110-95FD-441B-9811-AE78A5A06142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37C16DD6-4AEF-4226-9BB4-E576B07D7431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="1710" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,10 +36,10 @@
     <t>RECEIVING DATE</t>
   </si>
   <si>
-    <t>ISSUE DATE</t>
+    <t>STATUS</t>
   </si>
   <si>
-    <t>STATUS</t>
+    <t>INSP DATE</t>
   </si>
 </sst>
 </file>
@@ -410,10 +410,10 @@
         <v>0</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>